<commit_message>
Mise à jour page Seuils
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\seuils\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D65E88A6-A824-4724-B156-3A1CFEE5ADC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6568DB26-6BFF-4CA6-848A-9196866AB3EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
@@ -1235,7 +1235,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="14">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -1275,7 +1275,7 @@
         <v>14</v>
       </c>
       <c r="F10" s="14">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -1295,7 +1295,7 @@
         <v>15</v>
       </c>
       <c r="F11" s="14">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -1335,7 +1335,7 @@
         <v>17</v>
       </c>
       <c r="F13" s="14">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1475,7 +1475,7 @@
         <v>24</v>
       </c>
       <c r="F20" s="14">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1495,7 +1495,7 @@
         <v>25</v>
       </c>
       <c r="F21" s="14">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1815,7 +1815,7 @@
         <v>41</v>
       </c>
       <c r="F37" s="14">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1975,7 +1975,7 @@
         <v>49</v>
       </c>
       <c r="F45" s="14">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -2035,7 +2035,7 @@
         <v>52</v>
       </c>
       <c r="F48" s="14">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -2055,7 +2055,7 @@
         <v>53</v>
       </c>
       <c r="F49" s="14">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -2075,7 +2075,7 @@
         <v>54</v>
       </c>
       <c r="F50" s="14">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -2115,7 +2115,7 @@
         <v>56</v>
       </c>
       <c r="F52" s="14">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
@@ -2155,7 +2155,7 @@
         <v>58</v>
       </c>
       <c r="F54" s="14">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>